<commit_message>
Update hotwords-thieu.xlsx with new data
</commit_message>
<xml_diff>
--- a/data/asr-gold/hotwords-thieu.xlsx
+++ b/data/asr-gold/hotwords-thieu.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,13 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,9 +59,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -13849,9 +13857,9 @@
           <t>FLIGHT LEVEL (number)</t>
         </is>
       </c>
-      <c r="B584" t="inlineStr">
-        <is>
-          <t>Mức bay (số)</t>
+      <c r="B584" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mực bay (số)</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
@@ -13930,9 +13938,9 @@
           <t>CLIMB TO (level)</t>
         </is>
       </c>
-      <c r="B587" t="inlineStr">
-        <is>
-          <t>Lên (mức)</t>
+      <c r="B587" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lên độ cao(mức)</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
@@ -13957,9 +13965,9 @@
           <t>DESCEND TO (level)</t>
         </is>
       </c>
-      <c r="B588" t="inlineStr">
-        <is>
-          <t>Xuống (mức)</t>
+      <c r="B588" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hạ độ cao xuống (mức)</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
@@ -14011,9 +14019,9 @@
           <t>CLIMB TO AND MAINTAIN BLOCK (level) TO (level)</t>
         </is>
       </c>
-      <c r="B590" t="inlineStr">
-        <is>
-          <t>Lên và giữ khối mức (mức) đến (mức)</t>
+      <c r="B590" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lên và giữ mực bay (mức) đến (mức)</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
@@ -14038,9 +14046,9 @@
           <t>DESCEND TO AND MAINTAIN BLOCK (level) TO (level)</t>
         </is>
       </c>
-      <c r="B591" t="inlineStr">
-        <is>
-          <t>Xuống và giữ khối mức (mức) đến (mức)</t>
+      <c r="B591" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Xuống và giữ mực bay (mức) đến (mức)</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
@@ -14065,9 +14073,9 @@
           <t>STOP CLIMB AT (level)</t>
         </is>
       </c>
-      <c r="B592" t="inlineStr">
-        <is>
-          <t>Dừng leo tại (mức)</t>
+      <c r="B592" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dừng lên độ cao tại (mực bay hoặc số)</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
@@ -14092,9 +14100,9 @@
           <t>STOP DESCENT AT (level)</t>
         </is>
       </c>
-      <c r="B593" t="inlineStr">
-        <is>
-          <t>Dừng hạ tại (mức)</t>
+      <c r="B593" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dừng hạ độ cao tại (mức)</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -14173,9 +14181,9 @@
           <t>CLIMB AT (number) FEET PER MINUTE OR GREATER</t>
         </is>
       </c>
-      <c r="B596" t="inlineStr">
-        <is>
-          <t>Leo với tốc độ thẳng đứng (số) feet/phút hoặc lớn hơn</t>
+      <c r="B596" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leo với tốc độ  (số) feet/phút hoặc lớn hơn</t>
         </is>
       </c>
       <c r="C596" t="inlineStr">
@@ -14200,9 +14208,9 @@
           <t>DESCEND AT (number) FEET PER MINUTE OR GREATER</t>
         </is>
       </c>
-      <c r="B597" t="inlineStr">
-        <is>
-          <t>Hạ với tốc độ thẳng đứng (số) feet/phút hoặc lớn hơn</t>
+      <c r="B597" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hạ với tốc độ (số) feet/phút hoặc lớn hơn</t>
         </is>
       </c>
       <c r="C597" t="inlineStr">
@@ -14875,9 +14883,9 @@
           <t>SQUAWK (code)</t>
         </is>
       </c>
-      <c r="B622" t="inlineStr">
-        <is>
-          <t>Đặt mã đáp (mã)</t>
+      <c r="B622" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đặt mã (mã)</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
@@ -14902,9 +14910,9 @@
           <t>REDUCE SPEED TO (number) KNOTS</t>
         </is>
       </c>
-      <c r="B623" t="inlineStr">
-        <is>
-          <t>Giảm tốc độ đến (số) knots</t>
+      <c r="B623" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giảm tốc độ còn (số) knots</t>
         </is>
       </c>
       <c r="C623" t="inlineStr">
@@ -15307,9 +15315,9 @@
           <t>CLEARED VISUAL APPROACH RUNWAY (number)</t>
         </is>
       </c>
-      <c r="B638" t="inlineStr">
-        <is>
-          <t>Được phép tiếp cận nhìn thấy đường CHC (số)</t>
+      <c r="B638" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Được phép tiếp cận bằng mắt đường CHC (số)</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -15496,9 +15504,9 @@
           <t>JOIN LEFT DOWNWIND RUNWAY (number)</t>
         </is>
       </c>
-      <c r="B645" t="inlineStr">
-        <is>
-          <t>Nhập chân gió xuôi trái đường CHC (số)</t>
+      <c r="B645" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tiến nhập cạnh 3 bên trái đường CHC (số)</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -15523,9 +15531,9 @@
           <t>JOIN RIGHT DOWNWIND RUNWAY (number)</t>
         </is>
       </c>
-      <c r="B646" t="inlineStr">
-        <is>
-          <t>Nhập chân gió xuôi phải đường CHC (số)</t>
+      <c r="B646" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tiến nhập cạnh 3 bên phải đường CHC (số)</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -19217,9 +19225,9 @@
       </c>
     </row>
     <row r="783">
-      <c r="A783" t="inlineStr">
-        <is>
-          <t>Saigon Approach</t>
+      <c r="A783" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tan Son Nhat Approach</t>
         </is>
       </c>
       <c r="B783" t="inlineStr">
@@ -19276,9 +19284,9 @@
           <t>November</t>
         </is>
       </c>
-      <c r="B785" t="inlineStr">
-        <is>
-          <t>đường lăn N — Nội Bài</t>
+      <c r="B785" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn N </t>
         </is>
       </c>
       <c r="C785" t="inlineStr">
@@ -19303,9 +19311,9 @@
           <t>November One</t>
         </is>
       </c>
-      <c r="B786" t="inlineStr">
-        <is>
-          <t>đường lăn N1 — Nội Bài</t>
+      <c r="B786" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn N1</t>
         </is>
       </c>
       <c r="C786" t="inlineStr">
@@ -19330,9 +19338,9 @@
           <t>November Two</t>
         </is>
       </c>
-      <c r="B787" t="inlineStr">
-        <is>
-          <t>đường lăn N2 — Nội Bài</t>
+      <c r="B787" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn N2 </t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
@@ -19357,9 +19365,9 @@
           <t>November Three</t>
         </is>
       </c>
-      <c r="B788" t="inlineStr">
-        <is>
-          <t>đường lăn N3 — Nội Bài</t>
+      <c r="B788" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn N3 </t>
         </is>
       </c>
       <c r="C788" t="inlineStr">
@@ -19384,9 +19392,9 @@
           <t>November Four</t>
         </is>
       </c>
-      <c r="B789" t="inlineStr">
-        <is>
-          <t>đường lăn N4 — Nội Bài</t>
+      <c r="B789" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn N4 </t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
@@ -19411,9 +19419,9 @@
           <t>November Five</t>
         </is>
       </c>
-      <c r="B790" t="inlineStr">
-        <is>
-          <t>đường lăn N5 — Nội Bài</t>
+      <c r="B790" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn N5 </t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
@@ -19438,9 +19446,9 @@
           <t>Papa Three</t>
         </is>
       </c>
-      <c r="B791" t="inlineStr">
-        <is>
-          <t>đường lăn P3 — Nội Bài</t>
+      <c r="B791" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P3 </t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
@@ -19465,9 +19473,9 @@
           <t>Papa Four</t>
         </is>
       </c>
-      <c r="B792" t="inlineStr">
-        <is>
-          <t>đường lăn P4 — Nội Bài</t>
+      <c r="B792" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P4 </t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
@@ -19492,9 +19500,9 @@
           <t>Papa Five</t>
         </is>
       </c>
-      <c r="B793" t="inlineStr">
-        <is>
-          <t>đường lăn P5 — Nội Bài</t>
+      <c r="B793" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P5 </t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
@@ -19519,9 +19527,9 @@
           <t>Papa Six</t>
         </is>
       </c>
-      <c r="B794" t="inlineStr">
-        <is>
-          <t>đường lăn P6 — Nội Bài</t>
+      <c r="B794" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P6 </t>
         </is>
       </c>
       <c r="C794" t="inlineStr">
@@ -19546,9 +19554,9 @@
           <t>Papa Seven</t>
         </is>
       </c>
-      <c r="B795" t="inlineStr">
-        <is>
-          <t>đường lăn P7 — Nội Bài</t>
+      <c r="B795" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P7 </t>
         </is>
       </c>
       <c r="C795" t="inlineStr">
@@ -19573,9 +19581,9 @@
           <t>Papa Eight</t>
         </is>
       </c>
-      <c r="B796" t="inlineStr">
-        <is>
-          <t>đường lăn P8 — Nội Bài</t>
+      <c r="B796" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P8 </t>
         </is>
       </c>
       <c r="C796" t="inlineStr">
@@ -19600,9 +19608,9 @@
           <t>Papa Nine</t>
         </is>
       </c>
-      <c r="B797" t="inlineStr">
-        <is>
-          <t>đường lăn P9 — Nội Bài</t>
+      <c r="B797" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P9 </t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
@@ -19627,9 +19635,9 @@
           <t>Sierra</t>
         </is>
       </c>
-      <c r="B798" t="inlineStr">
-        <is>
-          <t>đường lăn S — Nội Bài</t>
+      <c r="B798" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S </t>
         </is>
       </c>
       <c r="C798" t="inlineStr">
@@ -19654,9 +19662,9 @@
           <t>Sierra One</t>
         </is>
       </c>
-      <c r="B799" t="inlineStr">
-        <is>
-          <t>đường lăn S1 — Nội Bài</t>
+      <c r="B799" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S1 </t>
         </is>
       </c>
       <c r="C799" t="inlineStr">
@@ -19681,9 +19689,9 @@
           <t>Sierra Three</t>
         </is>
       </c>
-      <c r="B800" t="inlineStr">
-        <is>
-          <t>đường lăn S3 — Nội Bài</t>
+      <c r="B800" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S3 </t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
@@ -19708,9 +19716,9 @@
           <t>Sierra One Zero</t>
         </is>
       </c>
-      <c r="B801" t="inlineStr">
-        <is>
-          <t>đường lăn S10 — Nội Bài</t>
+      <c r="B801" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S10 </t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
@@ -19735,9 +19743,9 @@
           <t>Sierra Four</t>
         </is>
       </c>
-      <c r="B802" t="inlineStr">
-        <is>
-          <t>đường lăn S4 — Nội Bài</t>
+      <c r="B802" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S4 </t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
@@ -19762,9 +19770,9 @@
           <t>Sierra Five</t>
         </is>
       </c>
-      <c r="B803" t="inlineStr">
-        <is>
-          <t>đường lăn S5 — Nội Bài</t>
+      <c r="B803" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S5 </t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
@@ -19789,9 +19797,9 @@
           <t>Sierra Six</t>
         </is>
       </c>
-      <c r="B804" t="inlineStr">
-        <is>
-          <t>đường lăn S6 — Nội Bài</t>
+      <c r="B804" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S6 </t>
         </is>
       </c>
       <c r="C804" t="inlineStr">
@@ -19816,9 +19824,9 @@
           <t>Sierra Seven</t>
         </is>
       </c>
-      <c r="B805" t="inlineStr">
-        <is>
-          <t>đường lăn S7 — Nội Bài</t>
+      <c r="B805" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S7 </t>
         </is>
       </c>
       <c r="C805" t="inlineStr">
@@ -19843,9 +19851,9 @@
           <t>Sierra Eight</t>
         </is>
       </c>
-      <c r="B806" t="inlineStr">
-        <is>
-          <t>đường lăn S8 — Nội Bài</t>
+      <c r="B806" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S8 </t>
         </is>
       </c>
       <c r="C806" t="inlineStr">
@@ -19870,9 +19878,9 @@
           <t>Sierra Nine</t>
         </is>
       </c>
-      <c r="B807" t="inlineStr">
-        <is>
-          <t>đường lăn S9 — Nội Bài</t>
+      <c r="B807" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn S9 </t>
         </is>
       </c>
       <c r="C807" t="inlineStr">
@@ -19897,9 +19905,9 @@
           <t>Victor</t>
         </is>
       </c>
-      <c r="B808" t="inlineStr">
-        <is>
-          <t>đường lăn V — Nội Bài</t>
+      <c r="B808" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V </t>
         </is>
       </c>
       <c r="C808" t="inlineStr">
@@ -19924,9 +19932,9 @@
           <t>Victor One</t>
         </is>
       </c>
-      <c r="B809" t="inlineStr">
-        <is>
-          <t>đường lăn V1 — Nội Bài</t>
+      <c r="B809" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V1</t>
         </is>
       </c>
       <c r="C809" t="inlineStr">
@@ -19951,9 +19959,9 @@
           <t>Victor Seven</t>
         </is>
       </c>
-      <c r="B810" t="inlineStr">
-        <is>
-          <t>đường lăn V7 — Nội Bài</t>
+      <c r="B810" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V7</t>
         </is>
       </c>
       <c r="C810" t="inlineStr">
@@ -19978,9 +19986,9 @@
           <t>Victor Eight</t>
         </is>
       </c>
-      <c r="B811" t="inlineStr">
-        <is>
-          <t>đường lăn V8 — Nội Bài</t>
+      <c r="B811" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V8</t>
         </is>
       </c>
       <c r="C811" t="inlineStr">
@@ -20005,9 +20013,9 @@
           <t>Victor Two</t>
         </is>
       </c>
-      <c r="B812" t="inlineStr">
-        <is>
-          <t>đường lăn V2 — Nội Bài</t>
+      <c r="B812" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V2</t>
         </is>
       </c>
       <c r="C812" t="inlineStr">
@@ -20032,9 +20040,9 @@
           <t>Victor Three</t>
         </is>
       </c>
-      <c r="B813" t="inlineStr">
-        <is>
-          <t>đường lăn V3 — Nội Bài</t>
+      <c r="B813" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V3</t>
         </is>
       </c>
       <c r="C813" t="inlineStr">
@@ -20059,9 +20067,9 @@
           <t>Victor Four</t>
         </is>
       </c>
-      <c r="B814" t="inlineStr">
-        <is>
-          <t>đường lăn V4 — Nội Bài</t>
+      <c r="B814" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V4</t>
         </is>
       </c>
       <c r="C814" t="inlineStr">
@@ -20086,9 +20094,9 @@
           <t>Victor Five</t>
         </is>
       </c>
-      <c r="B815" t="inlineStr">
-        <is>
-          <t>đường lăn V5 — Nội Bài</t>
+      <c r="B815" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V5</t>
         </is>
       </c>
       <c r="C815" t="inlineStr">
@@ -20113,9 +20121,9 @@
           <t>Victor Six</t>
         </is>
       </c>
-      <c r="B816" t="inlineStr">
-        <is>
-          <t>đường lăn V6 — Nội Bài</t>
+      <c r="B816" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V6</t>
         </is>
       </c>
       <c r="C816" t="inlineStr">
@@ -20140,9 +20148,9 @@
           <t>Victor Nine</t>
         </is>
       </c>
-      <c r="B817" t="inlineStr">
-        <is>
-          <t>đường lăn V9 — Nội Bài</t>
+      <c r="B817" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn V9</t>
         </is>
       </c>
       <c r="C817" t="inlineStr">
@@ -20167,9 +20175,9 @@
           <t>Papa One</t>
         </is>
       </c>
-      <c r="B818" t="inlineStr">
-        <is>
-          <t>đường lăn P1 — Tân Sơn Nhất</t>
+      <c r="B818" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P1</t>
         </is>
       </c>
       <c r="C818" t="inlineStr">
@@ -20194,9 +20202,9 @@
           <t>Papa Two</t>
         </is>
       </c>
-      <c r="B819" t="inlineStr">
-        <is>
-          <t>đường lăn P2 — Tân Sơn Nhất</t>
+      <c r="B819" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn P2</t>
         </is>
       </c>
       <c r="C819" t="inlineStr">
@@ -20221,9 +20229,9 @@
           <t>Zulu</t>
         </is>
       </c>
-      <c r="B820" t="inlineStr">
-        <is>
-          <t>đường lăn Z — Tân Sơn Nhất</t>
+      <c r="B820" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn Z</t>
         </is>
       </c>
       <c r="C820" t="inlineStr">
@@ -20248,9 +20256,9 @@
           <t>Zulu One</t>
         </is>
       </c>
-      <c r="B821" t="inlineStr">
-        <is>
-          <t>đường lăn Z1 — Tân Sơn Nhất</t>
+      <c r="B821" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn Z1 </t>
         </is>
       </c>
       <c r="C821" t="inlineStr">
@@ -20275,9 +20283,9 @@
           <t>Zulu Six</t>
         </is>
       </c>
-      <c r="B822" t="inlineStr">
-        <is>
-          <t>đường lăn Z6 — Tân Sơn Nhất</t>
+      <c r="B822" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn Z6</t>
         </is>
       </c>
       <c r="C822" t="inlineStr">
@@ -20302,9 +20310,9 @@
           <t>Zulu Seven</t>
         </is>
       </c>
-      <c r="B823" t="inlineStr">
-        <is>
-          <t>đường lăn Z7 — Tân Sơn Nhất</t>
+      <c r="B823" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn Z7</t>
         </is>
       </c>
       <c r="C823" t="inlineStr">
@@ -20329,9 +20337,9 @@
           <t>Echo</t>
         </is>
       </c>
-      <c r="B824" t="inlineStr">
-        <is>
-          <t>đường lăn E — Đà Nẵng</t>
+      <c r="B824" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn E</t>
         </is>
       </c>
       <c r="C824" t="inlineStr">
@@ -20356,9 +20364,9 @@
           <t>Echo One</t>
         </is>
       </c>
-      <c r="B825" t="inlineStr">
-        <is>
-          <t>đường lăn E1 — Đà Nẵng</t>
+      <c r="B825" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn E1</t>
         </is>
       </c>
       <c r="C825" t="inlineStr">
@@ -20383,9 +20391,9 @@
           <t>Echo Two</t>
         </is>
       </c>
-      <c r="B826" t="inlineStr">
-        <is>
-          <t>đường lăn E2 — Đà Nẵng</t>
+      <c r="B826" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn E2 </t>
         </is>
       </c>
       <c r="C826" t="inlineStr">
@@ -20410,9 +20418,9 @@
           <t>Echo Three</t>
         </is>
       </c>
-      <c r="B827" t="inlineStr">
-        <is>
-          <t>đường lăn E3 — Đà Nẵng</t>
+      <c r="B827" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn E3</t>
         </is>
       </c>
       <c r="C827" t="inlineStr">
@@ -20437,9 +20445,9 @@
           <t>Echo Four</t>
         </is>
       </c>
-      <c r="B828" t="inlineStr">
-        <is>
-          <t>đường lăn E4 — Đà Nẵng</t>
+      <c r="B828" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn E4</t>
         </is>
       </c>
       <c r="C828" t="inlineStr">
@@ -20464,9 +20472,9 @@
           <t>Echo Six</t>
         </is>
       </c>
-      <c r="B829" t="inlineStr">
-        <is>
-          <t>đường lăn E6 — Đà Nẵng</t>
+      <c r="B829" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn E5</t>
         </is>
       </c>
       <c r="C829" t="inlineStr">
@@ -20491,9 +20499,9 @@
           <t>Echo Seven</t>
         </is>
       </c>
-      <c r="B830" t="inlineStr">
-        <is>
-          <t>đường lăn E7 — Đà Nẵng</t>
+      <c r="B830" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">đường lăn E6</t>
         </is>
       </c>
       <c r="C830" t="inlineStr">

</xml_diff>